<commit_message>
DATA: Corri mnm.py para ARG, USA y ENG para predecir proximos partidos y probar cambios recien implementados en mnm.py
</commit_message>
<xml_diff>
--- a/data/argentina/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
+++ b/data/argentina/p6_deployment/data_preparation/clean_data/df_match_cleaned.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:O16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,45 +507,45 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>noM4eJv9</t>
+          <t>fotMKZ7K</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45506.83333333334</v>
+        <v>45513.625</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">espinoza f 
+          <t xml:space="preserve">mastrangelo h 
   arg </t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">estadio marcelo bielsa
-  rosario </t>
+          <t xml:space="preserve">estadio guillermo laza
+  buenos aires </t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>42000</v>
+        <v>3000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>6gMiRHVj</t>
+          <t>2iZ4q0z6</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>newells old boys</t>
+          <t>dep  riestra</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>p2SkCHXs</t>
+          <t>Y9yh1J7G</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>estudiantes l p</t>
+          <t>lanus</t>
         </is>
       </c>
       <c r="J2" t="n">
@@ -574,45 +574,45 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>nkx6zI2q</t>
+          <t>YHCv8dOE</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45507.625</v>
+        <v>45513.6875</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">gariano a 
+          <t xml:space="preserve">trucco s 
   arg </t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">estadio malvinas argentinas
-  mendoza </t>
+          <t xml:space="preserve">claudio fabian tapia
+  barracas </t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>42000</v>
+        <v>4400</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>tUAxIm6l</t>
+          <t>hW08cP6J</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>godoy cruz</t>
+          <t>barracas central</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>QuxS0ahA</t>
+          <t>bkDdeAvA</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>argentinos jrs</t>
+          <t>talleres cordoba</t>
         </is>
       </c>
       <c r="J3" t="n">
@@ -641,45 +641,45 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>pdWqnF1e</t>
+          <t>llkWcC07</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45507.625</v>
+        <v>45513.79166666666</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">lamolina n 
+          <t xml:space="preserve">herrera d 
   arg </t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">estadio jose amalfitani
-  buenos aires </t>
+          <t xml:space="preserve">estadio julio cesar villagra
+  cordoba </t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>49540</v>
+        <v>34830</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>UsCR8gFd</t>
+          <t>Amzaty2s</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>velez sarsfield</t>
+          <t>belgrano</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Gdfv0Zsh</t>
+          <t>lr2YMkTK</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>defensa y justicia</t>
+          <t>union de santa fe</t>
         </is>
       </c>
       <c r="J4" t="n">
@@ -708,45 +708,45 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>vq1qlyXr</t>
+          <t>hMeNaYVf</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>45507.71875</v>
+        <v>45513.875</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">herrera d 
+          <t xml:space="preserve">arasa n 
   arg </t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">estadio mario alberto kempes
-  cordoba </t>
+          <t xml:space="preserve">estadio juan domingo peron
+  avellaneda </t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>57000</v>
+        <v>61000</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>bkDdeAvA</t>
+          <t>OhapHPm9</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>talleres cordoba</t>
+          <t>racing club</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>8G45bXRA</t>
+          <t>jiDN9Zaj</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>instituto</t>
+          <t>gimnasia l p</t>
         </is>
       </c>
       <c r="J5" t="n">
@@ -775,45 +775,45 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>U9B9fwfF</t>
+          <t>trGn6zgR</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>45507.80208333334</v>
+        <v>45514.60416666666</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">mastrangelo h 
+          <t xml:space="preserve">rey hilfer l 
   arg </t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">estadio libertadores de america
-  avellaneda </t>
+          <t xml:space="preserve">estadio pedro bidegain
+  buenos aires </t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>48069</v>
+        <v>47964</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>UVatI5Y2</t>
+          <t>ju1xJoJd</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>independiente</t>
+          <t>san lorenzo</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>ju1xJoJd</t>
+          <t>KpqpxWko</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>san lorenzo</t>
+          <t>atl  tucuman</t>
         </is>
       </c>
       <c r="J6" t="n">
@@ -842,45 +842,45 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>KvUIXFn2</t>
+          <t>badJ0EGl</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>45507.85416666666</v>
+        <v>45514.6875</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">tello f 
+          <t xml:space="preserve">ramirez n 
   arg </t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">estadio tomas adolfo duco
-  buenos aires </t>
+          <t xml:space="preserve">estadio gigante de arroyito
+  rosario </t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>48314</v>
+        <v>46955</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>xd3lGq3F</t>
+          <t>4QmJ2LNc</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>huracan</t>
+          <t>rosario central</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>OhapHPm9</t>
+          <t>6gMiRHVj</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>racing club</t>
+          <t>newells old boys</t>
         </is>
       </c>
       <c r="J7" t="n">
@@ -909,45 +909,45 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>bPuAZyIk</t>
+          <t>2iHr7GwL</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>45508.625</v>
+        <v>45514.78125</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ramirez n 
+          <t xml:space="preserve">tello f 
   arg </t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">estadio eva peron
-  junin </t>
+          <t xml:space="preserve">estadio juan bautista gargantini
+  mendoza </t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>22000</v>
+        <v>24000</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>KQ6kGfyc</t>
+          <t>Eg51aDC4</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>sarmiento junin</t>
+          <t>ind  rivadavia</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Amzaty2s</t>
+          <t>hMrWAFH0</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>belgrano</t>
+          <t>boca juniors</t>
         </is>
       </c>
       <c r="J8" t="n">
@@ -976,45 +976,45 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>tlVEYeXe</t>
+          <t>WCfRbho1</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>45508.625</v>
+        <v>45514.85416666666</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">echavarria p 
+          <t xml:space="preserve">echenique f 
   arg </t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">estadio 15 de abril
-  santa fe </t>
+          <t xml:space="preserve">estadio monumental
+  buenos aires </t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>27358</v>
+        <v>84567</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>lr2YMkTK</t>
+          <t>EVqSBe2f</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>union de santa fe</t>
+          <t>river plate</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>EVqSBe2f</t>
+          <t>xd3lGq3F</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>river plate</t>
+          <t>huracan</t>
         </is>
       </c>
       <c r="J9" t="n">
@@ -1043,45 +1043,45 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>xzFHhHOR</t>
+          <t>vJVmoZG1</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>45508.72916666666</v>
+        <v>45515.625</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">echenique f 
+          <t xml:space="preserve">espinoza f 
   arg </t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">estadio alberto j  armando
-  buenos aires </t>
+          <t xml:space="preserve">estadio unico madre de ciudades
+  santiago del estero </t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>57200</v>
+        <v>42000</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>hMrWAFH0</t>
+          <t>0dHZReql</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>boca juniors</t>
+          <t>central cordoba</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>hW08cP6J</t>
+          <t>Gdfv0Zsh</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>barracas central</t>
+          <t>defensa y justicia</t>
         </is>
       </c>
       <c r="J10" t="n">
@@ -1110,45 +1110,45 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>rDFDgc9L</t>
+          <t>fRDz9x98</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>45508.83333333334</v>
+        <v>45515.625</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">arasa n 
+          <t xml:space="preserve">balino j 
   arg </t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">estadio monumental jose fierro
-  tucuman </t>
+          <t xml:space="preserve">estadio presidente peron
+  cordoba </t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>35200</v>
+        <v>26000</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>KpqpxWko</t>
+          <t>8G45bXRA</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>atl  tucuman</t>
+          <t>instituto</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Eg51aDC4</t>
+          <t>80MMdBdN</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>ind  rivadavia</t>
+          <t>platense</t>
         </is>
       </c>
       <c r="J11" t="n">
@@ -1177,11 +1177,11 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>U9kvubfS</t>
+          <t>hMZipgW7</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>45508.83333333334</v>
+        <v>45515.72916666666</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1191,31 +1191,31 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">estadio ciudad de lanus – nestor diaz perez
-  lanus </t>
+          <t xml:space="preserve">estadio florencio sola
+  buenos aires </t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>47090</v>
+        <v>34902</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Y9yh1J7G</t>
+          <t>GIb40wNM</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>lanus</t>
+          <t>banfield</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>nkwO1uw4</t>
+          <t>UsCR8gFd</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>tigre</t>
+          <t>velez sarsfield</t>
         </is>
       </c>
       <c r="J12" t="n">
@@ -1244,45 +1244,45 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>jJjztvuM</t>
+          <t>nPhF1f1r</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>45509.60416666666</v>
+        <v>45515.83333333334</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">rey hilfer l 
+          <t xml:space="preserve">zunino s 
   arg </t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">estadio guillermo laza
-  buenos aires </t>
+          <t xml:space="preserve">estadio jorge luis hirschi
+  la plata </t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>3000</v>
+        <v>32530</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2iZ4q0z6</t>
+          <t>p2SkCHXs</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>dep  riestra</t>
+          <t>estudiantes l p</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>0dHZReql</t>
+          <t>UVatI5Y2</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>central cordoba</t>
+          <t>independiente</t>
         </is>
       </c>
       <c r="J13" t="n">
@@ -1311,45 +1311,40 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>8fN0daP2</t>
+          <t>trxILFhE</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>45509.70833333334</v>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zunino s 
-  arg </t>
-        </is>
-      </c>
+        <v>45516.79166666666</v>
+      </c>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">estadio juan carmelo zerillo
-  la plata </t>
+          <t xml:space="preserve">estadio jose dellagiovanna
+  buenos aires </t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>21500</v>
+        <v>26282</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>jiDN9Zaj</t>
+          <t>nkwO1uw4</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>gimnasia l p</t>
+          <t>tigre</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>4QmJ2LNc</t>
+          <t>tUAxIm6l</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>rosario central</t>
+          <t>godoy cruz</t>
         </is>
       </c>
       <c r="J14" t="n">
@@ -1378,55 +1373,50 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>65Xumenk</t>
+          <t>Y9EiyTMr</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>45509.83333333334</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">penel a 
-  arg </t>
-        </is>
-      </c>
+        <v>45518.79166666666</v>
+      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">estadio ciudad de vicente lopez
-  buenos aires </t>
+          <t xml:space="preserve">estadio libertadores de america
+  avellaneda </t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>28530</v>
+        <v>48069</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>80MMdBdN</t>
+          <t>QuxS0ahA</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>platense</t>
+          <t>argentinos jrs</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>GIb40wNM</t>
+          <t>xd3lGq3F</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>banfield</t>
+          <t>huracan</t>
         </is>
       </c>
       <c r="J15" t="n">
         <v>6</v>
       </c>
       <c r="K15" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="L15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M15" t="n">
         <v>2024</v>
@@ -1438,57 +1428,57 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>liga profesional</t>
+          <t>copa argentina</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>SvlzcWFD</t>
+          <t>fgvPVMI8</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>45512.625</v>
+        <v>45519.70833333334</v>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">estadio diego armando maradona
-  buenos aires </t>
+          <t xml:space="preserve">estadio centenario ciudad de quilmes
+  quilmes </t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>26000</v>
+        <v>30200</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>QuxS0ahA</t>
+          <t>ABogdBtb</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>argentinos jrs</t>
+          <t>talleres  r e</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>KQ6kGfyc</t>
+          <t>GIb40wNM</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>sarmiento junin</t>
+          <t>banfield</t>
         </is>
       </c>
       <c r="J16" t="n">
         <v>6</v>
       </c>
       <c r="K16" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="L16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M16" t="n">
         <v>2024</v>
@@ -1499,68 +1489,6 @@
         </is>
       </c>
       <c r="O16" t="inlineStr">
-        <is>
-          <t>liga profesional</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>ngdGLTFj</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>45510.88194444445</v>
-      </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">estadio libertadores de america
-  avellaneda </t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>48069</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>ju1xJoJd</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>san lorenzo</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>UsCR8gFd</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>velez sarsfield</t>
-        </is>
-      </c>
-      <c r="J17" t="n">
-        <v>6</v>
-      </c>
-      <c r="K17" t="n">
-        <v>64</v>
-      </c>
-      <c r="L17" t="n">
-        <v>1</v>
-      </c>
-      <c r="M17" t="n">
-        <v>2024</v>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>argentina</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
         <is>
           <t>copa argentina</t>
         </is>

</xml_diff>